<commit_message>
docs: 更新 2019 上半年真题 2019-shang-2.xlsx
</commit_message>
<xml_diff>
--- a/docs/public/exam/2019-shang-2.xlsx
+++ b/docs/public/exam/2019-shang-2.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="15">
   <si>
     <t>序号</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t>公式题，需要推导。</t>
+  </si>
+  <si>
+    <t>概念题。</t>
   </si>
   <si>
     <t>D*</t>
@@ -1908,7 +1911,9 @@
         <f t="shared" si="0"/>
         <v>假</v>
       </c>
-      <c r="E30" s="9"/>
+      <c r="E30" s="9" t="s">
+        <v>8</v>
+      </c>
       <c r="F30" s="9"/>
     </row>
     <row r="31" ht="14.25" hidden="1" spans="1:6">
@@ -1942,7 +1947,9 @@
         <f t="shared" si="0"/>
         <v>假</v>
       </c>
-      <c r="E32" s="9"/>
+      <c r="E32" s="9" t="s">
+        <v>8</v>
+      </c>
       <c r="F32" s="9"/>
     </row>
     <row r="33" ht="14.25" hidden="1" spans="1:6">
@@ -2102,7 +2109,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="22" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C42" s="15" t="s">
         <v>5</v>
@@ -2613,7 +2620,7 @@
     </row>
     <row r="78" ht="13.85" spans="1:2">
       <c r="A78" s="9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B78" s="25">
         <f>COUNTA(B2:B74)</f>
@@ -2622,7 +2629,7 @@
     </row>
     <row r="79" ht="13.85" spans="1:3">
       <c r="A79" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B79" s="25">
         <f>COUNTIF(D4:D76,"真")</f>
@@ -2632,7 +2639,7 @@
     </row>
     <row r="80" ht="13.85" spans="1:3">
       <c r="A80" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B80" s="25">
         <f>B78-B79</f>
@@ -2642,10 +2649,10 @@
     </row>
     <row r="81" ht="13.85" spans="1:2">
       <c r="A81" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B81" s="17" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>